<commit_message>
Evento #1 registrado en reporte_2026-06-04.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-04.xlsx
+++ b/datos/excel/reporte_2026-06-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,51 @@
         <v>10699</v>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>15:56:41</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>320.31</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-19.49</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>593.8 Hz | 921.9 Hz | 1257.8 Hz</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2522</v>
+      </c>
+      <c r="J3" t="n">
+        <v>10409</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #2 registrado en reporte_2026-06-04.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-04.xlsx
+++ b/datos/excel/reporte_2026-06-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,6 +603,51 @@
         <v>10326</v>
       </c>
       <c r="K4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>16:01:52</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>484.38</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-9.359999999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>968.8 Hz | 1453.1 Hz | 1945.3 Hz</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>2506</v>
+      </c>
+      <c r="J5" t="n">
+        <v>58</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #3 registrado en reporte_2026-06-04.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-04.xlsx
+++ b/datos/excel/reporte_2026-06-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -738,6 +738,51 @@
         <v>61</v>
       </c>
       <c r="K7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>16:04:06</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>484.38</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-9.390000000000001</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>976.6 Hz | 1453.1 Hz | 1945.3 Hz</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>2555</v>
+      </c>
+      <c r="J8" t="n">
+        <v>60</v>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #4 registrado en reporte_2026-06-04.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-04.xlsx
+++ b/datos/excel/reporte_2026-06-04.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1598,6 +1598,51 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>16:37:36</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>328.12</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-22.23</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>648.4 Hz | 968.8 Hz | 1359.4 Hz</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>2506</v>
+      </c>
+      <c r="J27" t="n">
+        <v>82</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>